<commit_message>
Restore landing page and add category routes
</commit_message>
<xml_diff>
--- a/28082026. Total product on MiniApp.xlsx
+++ b/28082026. Total product on MiniApp.xlsx
@@ -5924,118 +5924,6 @@
       <c r="Y75" s="3"/>
       <c r="Z75" s="3"/>
     </row>
-    <row r="76" ht="14.25" customHeight="1">
-      <c r="A76" s="37">
-        <v>73.0</v>
-      </c>
-      <c r="B76" s="38" t="s">
-        <v>219</v>
-      </c>
-      <c r="C76" s="39" t="s">
-        <v>219</v>
-      </c>
-      <c r="D76" s="39" t="s">
-        <v>281</v>
-      </c>
-      <c r="E76" s="40" t="s">
-        <v>282</v>
-      </c>
-      <c r="F76" s="41"/>
-      <c r="G76" s="42">
-        <v>1.28295E7</v>
-      </c>
-      <c r="H76" s="39">
-        <v>1110000.0</v>
-      </c>
-      <c r="I76" s="39">
-        <v>590000.0</v>
-      </c>
-      <c r="J76" s="39">
-        <v>430000.0</v>
-      </c>
-      <c r="K76" s="43"/>
-      <c r="L76" s="38">
-        <v>1.28295E7</v>
-      </c>
-      <c r="M76" s="39">
-        <v>1.332E7</v>
-      </c>
-      <c r="N76" s="39">
-        <v>1.416E7</v>
-      </c>
-      <c r="O76" s="39">
-        <v>1.548E7</v>
-      </c>
-      <c r="P76" s="44" t="s">
-        <v>283</v>
-      </c>
-      <c r="Q76" s="3"/>
-      <c r="R76" s="3"/>
-      <c r="S76" s="3"/>
-      <c r="T76" s="3"/>
-      <c r="U76" s="3"/>
-      <c r="V76" s="3"/>
-      <c r="W76" s="3"/>
-      <c r="X76" s="3"/>
-      <c r="Y76" s="3"/>
-      <c r="Z76" s="3"/>
-    </row>
-    <row r="77" ht="14.25" customHeight="1">
-      <c r="A77" s="37">
-        <v>74.0</v>
-      </c>
-      <c r="B77" s="38" t="s">
-        <v>219</v>
-      </c>
-      <c r="C77" s="39" t="s">
-        <v>219</v>
-      </c>
-      <c r="D77" s="39" t="s">
-        <v>284</v>
-      </c>
-      <c r="E77" s="40" t="s">
-        <v>285</v>
-      </c>
-      <c r="F77" s="41"/>
-      <c r="G77" s="42">
-        <v>1.38195E7</v>
-      </c>
-      <c r="H77" s="39">
-        <v>1200000.0</v>
-      </c>
-      <c r="I77" s="39">
-        <v>630000.0</v>
-      </c>
-      <c r="J77" s="39">
-        <v>460000.0</v>
-      </c>
-      <c r="K77" s="43"/>
-      <c r="L77" s="38">
-        <v>1.38195E7</v>
-      </c>
-      <c r="M77" s="39">
-        <v>1.44E7</v>
-      </c>
-      <c r="N77" s="39">
-        <v>1.512E7</v>
-      </c>
-      <c r="O77" s="39">
-        <v>1.656E7</v>
-      </c>
-      <c r="P77" s="44" t="s">
-        <v>283</v>
-      </c>
-      <c r="Q77" s="3"/>
-      <c r="R77" s="3"/>
-      <c r="S77" s="3"/>
-      <c r="T77" s="3"/>
-      <c r="U77" s="3"/>
-      <c r="V77" s="3"/>
-      <c r="W77" s="3"/>
-      <c r="X77" s="3"/>
-      <c r="Y77" s="3"/>
-      <c r="Z77" s="3"/>
-    </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="19">
         <v>75.0</v>
@@ -6089,62 +5977,6 @@
       <c r="X78" s="3"/>
       <c r="Y78" s="3"/>
       <c r="Z78" s="3"/>
-    </row>
-    <row r="79" ht="14.25" customHeight="1">
-      <c r="A79" s="37">
-        <v>76.0</v>
-      </c>
-      <c r="B79" s="45" t="s">
-        <v>286</v>
-      </c>
-      <c r="C79" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="D79" s="46" t="s">
-        <v>291</v>
-      </c>
-      <c r="E79" s="47" t="s">
-        <v>292</v>
-      </c>
-      <c r="F79" s="41"/>
-      <c r="G79" s="48">
-        <v>2.15981E7</v>
-      </c>
-      <c r="H79" s="46">
-        <v>1870000.0</v>
-      </c>
-      <c r="I79" s="46">
-        <v>1000000.0</v>
-      </c>
-      <c r="J79" s="46">
-        <v>810000.0</v>
-      </c>
-      <c r="K79" s="43"/>
-      <c r="L79" s="45">
-        <v>2.15981E7</v>
-      </c>
-      <c r="M79" s="46">
-        <v>2.244E7</v>
-      </c>
-      <c r="N79" s="46">
-        <v>2.4E7</v>
-      </c>
-      <c r="O79" s="46">
-        <v>2.916E7</v>
-      </c>
-      <c r="P79" s="44" t="s">
-        <v>293</v>
-      </c>
-      <c r="Q79" s="3"/>
-      <c r="R79" s="3"/>
-      <c r="S79" s="3"/>
-      <c r="T79" s="3"/>
-      <c r="U79" s="3"/>
-      <c r="V79" s="3"/>
-      <c r="W79" s="3"/>
-      <c r="X79" s="3"/>
-      <c r="Y79" s="3"/>
-      <c r="Z79" s="3"/>
     </row>
     <row r="80" ht="14.25" customHeight="1">
       <c r="A80" s="19">
@@ -36665,118 +36497,6 @@
       <c r="Y82" s="3"/>
       <c r="Z82" s="3"/>
     </row>
-    <row r="83" ht="14.25" customHeight="1">
-      <c r="A83" s="53">
-        <v>73.0</v>
-      </c>
-      <c r="B83" s="54" t="s">
-        <v>219</v>
-      </c>
-      <c r="C83" s="55" t="s">
-        <v>219</v>
-      </c>
-      <c r="D83" s="55" t="s">
-        <v>281</v>
-      </c>
-      <c r="E83" s="55" t="s">
-        <v>282</v>
-      </c>
-      <c r="F83" s="56" t="s">
-        <v>283</v>
-      </c>
-      <c r="G83" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="H83" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="I83" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="J83" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="K83" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="L83" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="M83" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="N83" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="O83" s="3"/>
-      <c r="P83" s="3"/>
-      <c r="Q83" s="3"/>
-      <c r="R83" s="3"/>
-      <c r="S83" s="3"/>
-      <c r="T83" s="3"/>
-      <c r="U83" s="3"/>
-      <c r="V83" s="3"/>
-      <c r="W83" s="3"/>
-      <c r="X83" s="3"/>
-      <c r="Y83" s="3"/>
-      <c r="Z83" s="3"/>
-    </row>
-    <row r="84" ht="14.25" customHeight="1">
-      <c r="A84" s="53">
-        <v>74.0</v>
-      </c>
-      <c r="B84" s="54" t="s">
-        <v>219</v>
-      </c>
-      <c r="C84" s="55" t="s">
-        <v>219</v>
-      </c>
-      <c r="D84" s="55" t="s">
-        <v>284</v>
-      </c>
-      <c r="E84" s="55" t="s">
-        <v>285</v>
-      </c>
-      <c r="F84" s="56" t="s">
-        <v>283</v>
-      </c>
-      <c r="G84" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="H84" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="I84" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="J84" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="K84" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="L84" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="M84" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="N84" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="O84" s="3"/>
-      <c r="P84" s="3"/>
-      <c r="Q84" s="3"/>
-      <c r="R84" s="3"/>
-      <c r="S84" s="3"/>
-      <c r="T84" s="3"/>
-      <c r="U84" s="3"/>
-      <c r="V84" s="3"/>
-      <c r="W84" s="3"/>
-      <c r="X84" s="3"/>
-      <c r="Y84" s="3"/>
-      <c r="Z84" s="3"/>
-    </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="19">
         <v>75.0</v>
@@ -36830,62 +36550,6 @@
       <c r="X85" s="3"/>
       <c r="Y85" s="3"/>
       <c r="Z85" s="3"/>
-    </row>
-    <row r="86" ht="14.25" customHeight="1">
-      <c r="A86" s="53">
-        <v>76.0</v>
-      </c>
-      <c r="B86" s="59" t="s">
-        <v>286</v>
-      </c>
-      <c r="C86" s="60" t="s">
-        <v>290</v>
-      </c>
-      <c r="D86" s="60" t="s">
-        <v>291</v>
-      </c>
-      <c r="E86" s="60" t="s">
-        <v>292</v>
-      </c>
-      <c r="F86" s="56" t="s">
-        <v>293</v>
-      </c>
-      <c r="G86" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="H86" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="I86" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="J86" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="K86" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="L86" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="M86" s="57" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="N86" s="58" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
-      <c r="Q86" s="3"/>
-      <c r="R86" s="3"/>
-      <c r="S86" s="3"/>
-      <c r="T86" s="3"/>
-      <c r="U86" s="3"/>
-      <c r="V86" s="3"/>
-      <c r="W86" s="3"/>
-      <c r="X86" s="3"/>
-      <c r="Y86" s="3"/>
-      <c r="Z86" s="3"/>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="19">

</xml_diff>